<commit_message>
Re-run job search excluding defense and armament roles
- fresh LinkedIn search (24 keywords), 538 listings; 30 defense/armament
  roles excluded and listed in jobs/excluded_defense.json
- new ranking in jobs_ranked.md / jobs_ranked.xlsx (extra sheet with
  the excluded roles)
- new tailored CVs for Rychiger and Axpo; Rheinmetall and RUAG CVs removed;
  defense wording dropped from experience bullets

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWu37SZ914L6ncZ6mpAGWX
</commit_message>
<xml_diff>
--- a/jobs_ranked.xlsx
+++ b/jobs_ranked.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Stellen-Ranking" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ausgeschlossen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stellen-Ranking'!$A$4:$J$24</definedName>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +60,12 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="13"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -95,10 +102,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -115,6 +124,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -488,26 +505,26 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ranking passender Stellen in der Schweiz – Kornelia Kunstmann</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
+          <t>Ranking passender Stellen in der Schweiz – ohne Verteidigung/Rüstung – Kornelia Kunstmann</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Quelle: öffentliche LinkedIn-Jobsuche Schweiz (letzte 30 Tage), Stand 04.10.2026. Score 0–100: Rollen-Fit 35 · Branche 25 · Seniorität 15 · Muss-Kriterien 15 · Arbeitsweg ab Küssnacht am Rigi 10.</t>
+          <t>Quelle: öffentliche LinkedIn-Jobsuche Schweiz (letzte 30 Tage), Stand 04.10.2026; 538 Stellen gesammelt, 30 wegen Verteidigungs-/Rüstungsbezug ausgeschlossen (siehe Blatt 'Ausgeschlossen'). Score 0–100: Rollen-Fit 35 · Branche 25 · Seniorität 15 · Muss-Kriterien 15 · Arbeitsweg ab Küssnacht am Rigi 10.</t>
         </is>
       </c>
     </row>
@@ -568,46 +585,46 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Senior Project Manager Air Defence</t>
+          <t>Director, Project Management &amp; Operational Excellence, EMEA</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Rheinmetall</t>
+          <t>Johnson Controls</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Zürich-Oerlikon (~45 Min.)</t>
+          <t>Neuhausen am Rheinfall (~1h20)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Gesamtprojektleitung komplexer Flugabwehrsysteme; passt zu Luft- &amp; Raumfahrtstudium und DLR/ESA/maxon/RUAG; Spanisch von Vorteil, Deutsch/Englisch verhandlungssicher.</t>
+          <t>Director-Rolle: Operational Excellence, Prozessstandardisierung, Change Management und PM-Fähigkeiten in EMEA – deckt Top-Skills und Führungsstufe ab.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>IPMA-Zertifizierung erwünscht; mehrtägige Auslandsreisen.</t>
+          <t>Branche Gebäudetechnik (HVAC/Controls); ≥10 Jahre PM-Erfahrung verlangt (erfüllt).</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>cv/cv_rheinmetall_senior_pm_air_defence.pdf</t>
+          <t>cv/cv_johnson_controls_director_pm_opex.pdf</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4467181676/</t>
+          <t>https://www.linkedin.com/jobs/view/4465928173/</t>
         </is>
       </c>
     </row>
@@ -616,46 +633,46 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Project Manager UAV &amp; cUAV</t>
+          <t>Director Project Management</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>RUAG</t>
+          <t>Rychiger</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Emmen (~30 Min.)</t>
+          <t>Steffisburg BE (~1h30)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Business Development + Projektleitung: VBS-Drohnenprojekte gewinnen, Verhandlungen mit Partnern/Startups, Umsetzungsteam aufbauen; Luft- &amp; Raumfahrt-Abschluss gefragt; 7 Jahre RUAG Emmen.</t>
+          <t>Leitung von 10 Projektleitenden, internationale Maschinenbauprojekte, Multiprojekt-/Portfoliomanagement, Prozessstandards; KI-Affinität ausdrücklich gewünscht.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Schweizer Staatsangehörigkeit zwingend; Stufe unter der letzten Position.</t>
+          <t>Erfahrung im Maschinenbau bevorzugt; enge Zusammenarbeit mit CEO/Eigentümer; langer Arbeitsweg.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>cv/cv_ruag_pm_uav_cuav.pdf</t>
+          <t>cv/cv_rychiger_director_project_management.pdf</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4473985550/</t>
+          <t>https://www.linkedin.com/jobs/view/4465984677/</t>
         </is>
       </c>
     </row>
@@ -664,46 +681,46 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Director, Project Management &amp; Operational Excellence, EMEA</t>
+          <t>Process Excellence Manager</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Johnson Controls</t>
+          <t>Axpo Group</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Neuhausen am Rheinfall (~1h20)</t>
+          <t>Baden AG (~1h)</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Director-Rolle: Operational Excellence, Prozessstandardisierung, Change Management, PM-Fähigkeiten in EMEA – deckt Top-Skills und Führungsstufe ab; ausserhalb Verteidigung.</t>
+          <t>Process-Excellence-Initiativen, Operating Models, Governance, Organisationsentwicklung und Change – passt zu Business Process Manager und Lead Digital Transformation.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Branche Gebäudetechnik (HVAC/Controls); ≥10 Jahre PM-Erfahrung verlangt (erfüllt).</t>
+          <t>Celonis/Process Intelligence von Vorteil; keine Führungsrolle.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>cv/cv_johnson_controls_director_pm_opex.pdf</t>
+          <t>cv/cv_axpo_process_excellence_manager.pdf</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4465928173/</t>
+          <t>https://www.linkedin.com/jobs/view/4468664962/</t>
         </is>
       </c>
     </row>
@@ -712,42 +729,42 @@
         <v>4</v>
       </c>
       <c r="B8" s="7" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Program Manager Mission System (Defense &amp; High-Tech Mobility)</t>
+          <t>PMO &amp; Process Excellence Lead – MedTech R&amp;D</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Randstad (Kunde nicht genannt)</t>
+          <t>Consult (Kunde: MedTech-Firma)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Tägerwilen TG</t>
+          <t>Zug (~20 Min.)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Programmmanagement für Verteidigungs-Missionssysteme; Ingenieursabschluss, Englisch C1/C2, sehr gutes Deutsch.</t>
+          <t>PMO aufbauen, Portfolio-Governance, Reporting an Geschäftsleitung, Projektleitende coachen; sehr nah am Wohnort.</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Militärischer Hintergrund (Aufklärung) ist Plus; langer Arbeitsweg, 1–2 Tage Homeoffice; 20 % Reisen.</t>
+          <t>MedTech-/Life-Sciences-Hintergrund verlangt; PMP/IPMA von Vorteil.</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4464798329/</t>
+          <t>https://www.linkedin.com/jobs/view/4473237406/</t>
         </is>
       </c>
     </row>
@@ -756,42 +773,42 @@
         <v>5</v>
       </c>
       <c r="B9" s="7" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Sales Director Government Programs EMEA</t>
+          <t>Associate Director, Global Knowledge Management</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Jet Aviation</t>
+          <t>CSL</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Basel (vor Ort)</t>
+          <t>Glattbrugg ZH (~50 Min.)</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Business Development in Regierungs- und Sondermissions-Luftfahrt; Französisch/Deutsch/Spanisch von Vorteil.</t>
+          <t>Leitung globales Wissens- und Informationsmanagement mit Budget- und Personalverantwortung – Bezug zu Head Documentation und Digitalisierung.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>10+ Jahre Verteidigungsvertrieb verlangt; 50 % Reisen.</t>
+          <t>Pharma-Umfeld.</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4471449605/</t>
+          <t>https://www.linkedin.com/jobs/view/4475381683/</t>
         </is>
       </c>
     </row>
@@ -800,42 +817,42 @@
         <v>6</v>
       </c>
       <c r="B10" s="7" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Senior Project Manager (Aeronautics &amp; Defense)</t>
+          <t>AI Education &amp; Training Program Lead</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>fortil</t>
+          <t>ROSEN</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Genf</t>
+          <t>Stans NW (~30 Min.)</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Leitung von Luft- und Raumfahrtprogrammen von Entwicklung bis Industrialisierung.</t>
+          <t>KI-Befähigungsprogramm für ~4'500 Mitarbeitende: Change Management, Lernstandards, Workflow-Transformation; Claude-101-Zertifikat passt.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Weit entfernt vom Wohnort.</t>
+          <t>Eher Programm- als Linienführung.</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4470914271/</t>
+          <t>https://www.linkedin.com/jobs/view/4461229170/</t>
         </is>
       </c>
     </row>
@@ -844,42 +861,42 @@
         <v>7</v>
       </c>
       <c r="B11" s="7" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Technical Project Manager – Propulsion &amp; Pyrotechnics</t>
+          <t>Head of Operations</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Destinus</t>
+          <t>Novasina AG</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Zürich</t>
+          <t>Lachen SZ (~45 Min.)</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Programmleitung Raumfahrt-Hardware; Scale-up baut PM-Funktion auf.</t>
+          <t>Präzisionssensorik; Gesamtverantwortung Operations mit 13 MA; Operational Excellence.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Eher junior ausgeschrieben (3–6 Jahre).</t>
+          <t>Praktische Produktionserfahrung (Elektronik/SMD) zwingend.</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4473710743/</t>
+          <t>https://www.linkedin.com/jobs/view/4470164152/</t>
         </is>
       </c>
     </row>
@@ -888,42 +905,42 @@
         <v>8</v>
       </c>
       <c r="B12" s="7" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Head of Operations</t>
+          <t>Senior Director, Global Head Transformation Advanced Synthesis</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Novasina AG</t>
+          <t>Lonza</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Lachen SZ (~45 Min.)</t>
+          <t>Basel (~1h15)</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Präzisionssensorik; Gesamtverantwortung Operations mit 13 MA; Operational Excellence.</t>
+          <t>Globale Transformations- und OpEx-Programme über mehrere Standorte; Digitalisierung in der Fertigung.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Praktische Produktionserfahrung (Elektronik/SMD) zwingend.</t>
+          <t>10+ Jahre Fertigung/Operations, Lean-Six-Sigma-Belt bevorzugt; Pharma.</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr"/>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4470164152/</t>
+          <t>https://www.linkedin.com/jobs/view/4473350562/</t>
         </is>
       </c>
     </row>
@@ -936,38 +953,38 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Manager Systems Excellence &amp; Operations Controls Europe</t>
+          <t>Continuous Improvement Manager</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Johnson Controls</t>
+          <t>Hitachi Energy</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Bassersdorf ZH</t>
+          <t>Zürich (~45 Min.)</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Schwesterrolle zu Rang 3; Operational Excellence &amp; Change Management.</t>
+          <t>Lean-Six-Sigma-Initiativen in der Fertigung, Coaching von Teams, Transformationsprojekte.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Eine Stufe tiefer als Rang 3.</t>
+          <t>Shopfloor-Fokus; Lean-Six-Sigma-Erfahrung erwartet.</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4469348819/</t>
+          <t>https://www.linkedin.com/jobs/view/4460326016/</t>
         </is>
       </c>
     </row>
@@ -976,42 +993,42 @@
         <v>10</v>
       </c>
       <c r="B14" s="7" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Head of International Order Management – DIA Supply Chain</t>
+          <t>Business Development Manager Industrial Heating</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Leister Group</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Rotkreuz (~20 Min.)</t>
+          <t>Kägiswil OW (~35 Min.)</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Führung von 10–25 MA; Fokus Operational Excellence; nahe am Wohnort.</t>
+          <t>Business Development für Industrie-Prozesswärme, neue Märkte und Partner – passt zu Senior BD Manager.</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Export-/Zoll- und SAP-Expertise verlangt.</t>
+          <t>Vertriebsfokus; Erfahrung mit Distributoren gefragt.</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr"/>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4460363813/</t>
+          <t>https://www.linkedin.com/jobs/view/4467310897/</t>
         </is>
       </c>
     </row>
@@ -1020,42 +1037,42 @@
         <v>11</v>
       </c>
       <c r="B15" s="7" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Head of S&amp;C Ground Thun</t>
+          <t>Senior Transformation Manager Solution Engineering</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>RUAG</t>
+          <t>Siemens SI</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Thun</t>
+          <t>Zug (~25 Min.)</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Business Development &amp; Key Account Management Verteidigung; Change Management.</t>
+          <t>Transformationsrolle mit Top-Management-Mandat; Engineering + Digitalisierung.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Schweizer Nationalität oder Ausweis C zwingend.</t>
+          <t>Gebäudeautomation/Brandschutz.</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4469362716/</t>
+          <t>https://www.linkedin.com/jobs/view/4471937078/</t>
         </is>
       </c>
     </row>
@@ -1064,38 +1081,42 @@
         <v>12</v>
       </c>
       <c r="B16" s="7" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Senior Transformation Manager Solution Engineering</t>
+          <t>Head of International Order Management – DIA Supply Chain</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Siemens SI</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Zug (~25 Min.)</t>
+          <t>Rotkreuz (~20 Min.)</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Transformationsrolle mit Top-Management-Mandat; passt zu Digital Transformation + Engineering.</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr"/>
+          <t>Führung von 10–25 MA; Operational Excellence; nah am Wohnort.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Export-/Zoll- und SAP-Expertise verlangt.</t>
+        </is>
+      </c>
       <c r="I16" s="7" t="inlineStr"/>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4471937078/</t>
+          <t>https://www.linkedin.com/jobs/view/4460363813/</t>
         </is>
       </c>
     </row>
@@ -1104,42 +1125,42 @@
         <v>13</v>
       </c>
       <c r="B17" s="7" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Business Developer Defense</t>
+          <t>Manager Systems Excellence &amp; Operations Controls Europe</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Tethys Robotics</t>
+          <t>Johnson Controls</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Schlieren ZH</t>
+          <t>Bassersdorf ZH</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>ETH-Spin-off; Business Development Verteidigung.</t>
+          <t>Schwesterrolle zu Rang 1; Operational Excellence &amp; Change Management.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Bestehendes Netzwerk zu NATO-/Rüstungseinkäufern nötig.</t>
+          <t>Eine Stufe tiefer als Rang 1.</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr"/>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4466651737/</t>
+          <t>https://www.linkedin.com/jobs/view/4469348819/</t>
         </is>
       </c>
     </row>
@@ -1148,38 +1169,42 @@
         <v>14</v>
       </c>
       <c r="B18" s="7" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Lean Industrialization Manager</t>
+          <t>Director Operational Excellence &amp; PMO – Microbial Operations</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Jet Aviation</t>
+          <t>Lonza</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Basel</t>
+          <t>Visp VS</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Lean &amp; Operational Excellence in Luftfahrt (MRO, Completions).</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr"/>
+          <t>Director OpEx &amp; PMO an einem grossen Produktionsstandort.</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Pharma; vor Ort in Visp (Umzug nötig).</t>
+        </is>
+      </c>
       <c r="I18" s="7" t="inlineStr"/>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4466321768/</t>
+          <t>https://www.linkedin.com/jobs/view/4434120666/</t>
         </is>
       </c>
     </row>
@@ -1188,42 +1213,42 @@
         <v>15</v>
       </c>
       <c r="B19" s="7" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Supply Chain Excellence Manager:in</t>
+          <t>Lean Industrialization Manager</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Jarusel Recruiting (Kunde nicht genannt)</t>
+          <t>Jet Aviation</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Raum Luzern</t>
+          <t>Basel</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Lean/Six-Sigma-Projekte in der Supply Chain; nahe am Wohnort.</t>
+          <t>Lean &amp; Operational Excellence in der zivilen Luftfahrt (MRO, VIP-Completions).</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Lean/Six-Sigma-Erfahrung verlangt.</t>
+          <t>Vor Ort in Basel.</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr"/>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4469742762/</t>
+          <t>https://www.linkedin.com/jobs/view/4466321768/</t>
         </is>
       </c>
     </row>
@@ -1232,42 +1257,42 @@
         <v>16</v>
       </c>
       <c r="B20" s="7" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Senior Documentation Manager</t>
+          <t>Knowledge and Information Manager</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Bachem</t>
+          <t>Sika</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Bubendorf BL</t>
+          <t>Widen AG</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Direkter Bezug zur Rolle Head Documentation.</t>
+          <t>Engineering-Dokumentenmanagement (EDMS) &amp; Wissensmanagement + Digitalisierung.</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>GMP-/Pharma-Erfahrung verlangt.</t>
+          <t>Fachrolle ohne Führung.</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr"/>
       <c r="J20" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4469737075/</t>
+          <t>https://www.linkedin.com/jobs/view/4472932047/</t>
         </is>
       </c>
     </row>
@@ -1276,38 +1301,42 @@
         <v>17</v>
       </c>
       <c r="B21" s="7" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Knowledge and Information Manager</t>
+          <t>Umwelt- und Nachhaltigkeitsmanager:in</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Sika</t>
+          <t>Zentralbahn (SBB)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Widen AG</t>
+          <t>Stansstad NW (~25 Min.)</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Engineering-Dokumentenmanagement (EDMS) &amp; Wissensmanagement + digitale Transformation.</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr"/>
+          <t>Umwelt- und Nachhaltigkeitsstrategie, Biodiversität – passt zum Interesse an regenerativem Design/Permakultur.</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Fachausbildung Umwelt/Nachhaltigkeit erwartet.</t>
+        </is>
+      </c>
       <c r="I21" s="7" t="inlineStr"/>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4472932047/</t>
+          <t>https://www.linkedin.com/jobs/view/4474724588/</t>
         </is>
       </c>
     </row>
@@ -1316,42 +1345,42 @@
         <v>18</v>
       </c>
       <c r="B22" s="7" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Team Leader Account Management</t>
+          <t>Supply Chain Excellence Manager:in</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Pilatus Aircraft</t>
+          <t>Jarusel Recruiting (Kunde nicht genannt)</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Stans (~30 Min.)</t>
+          <t>Raum Luzern</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>After-Sales für Regierungsluftfahrt; Teamführung.</t>
+          <t>Lean/Six-Sigma-Projekte in der Supply Chain; nah am Wohnort.</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>10 Jahre Luftfahrterfahrung verlangt.</t>
+          <t>Lean/Six-Sigma-Erfahrung verlangt.</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr"/>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4466805480/</t>
+          <t>https://www.linkedin.com/jobs/view/4469742762/</t>
         </is>
       </c>
     </row>
@@ -1360,38 +1389,42 @@
         <v>19</v>
       </c>
       <c r="B23" s="7" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Sr Manager PMO &amp; Project Management</t>
+          <t>Maintenance Project Engineer / Manager</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>J&amp;J MedTech</t>
+          <t>AMAC Aerospace</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Zug</t>
+          <t>Basel</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>EMEA-PMO-Leitung für das Distributionsnetz.</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr"/>
+          <t>Projektleitung Flugzeugwartung und Modifikationen (zivil, VIP).</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Part-145/Part-21-Kenntnisse gefragt.</t>
+        </is>
+      </c>
       <c r="I23" s="7" t="inlineStr"/>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4468553924/</t>
+          <t>https://www.linkedin.com/jobs/view/4389218897/</t>
         </is>
       </c>
     </row>
@@ -1400,43 +1433,47 @@
         <v>20</v>
       </c>
       <c r="B24" s="7" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Teamlead Procurement &amp; Supply Chain</t>
+          <t>Senior Documentation Manager</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Wingtra</t>
+          <t>Bachem</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Zürich</t>
+          <t>Bubendorf BL</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Drohnen-Scale-up; Führung eines 4er-Teams.</t>
-        </is>
-      </c>
-      <c r="H24" s="7" t="inlineStr"/>
+          <t>Direkter Bezug zur Rolle Head Documentation.</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>GMP-/Pharma-Erfahrung verlangt.</t>
+        </is>
+      </c>
       <c r="I24" s="7" t="inlineStr"/>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4468973766/</t>
+          <t>https://www.linkedin.com/jobs/view/4469737075/</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>Blau hinterlegt: Top 3 – dafür liegen zugeschnittene Lebensläufe im Ordner cv/.</t>
         </is>
@@ -1471,4 +1508,901 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Ausgeschlossene Stellen (Verteidigung / Rüstung)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Stelle</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Firma</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Ort</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Grund</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Praticante universitario/a Trasformazione e innovazione Difesa</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Bundesverwaltung</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Bern, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Praktikum 'Trasformazione e innovazione Difesa' (Verteidigung)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4466868905/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Assembly &amp; Integration Technician</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Destinus</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Lucerne, Lucerne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4466040981/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Junior Buyer</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Destinus</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Payerne, Vaud, Switzerland</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4471472172/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Senior Propulsion Engineer (SRM)</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Destinus</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Payerne, Vaud, Switzerland</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4471439242/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Technical Project Manager - Propulsion &amp; Pyrotechnics</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Destinus</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4473710743/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Technical Project Manager - Propulsion &amp; Pyrotechnics</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Destinus</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Payerne, Vaud, Switzerland</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4473722052/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Capoprogetto Munizioni di grosso calibro</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Federal Office for Defence Procurement armasuisse</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Bern, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4465190832/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Projektleiter/-in für grosskalibrige Munition</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Federal Office for Defence Procurement armasuisse</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Bern, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464863487/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Computer Vision Engineer (VIO)</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Harmattan AI</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Lausanne, Vaud, Switzerland</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4472269161/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Director of Engineering - Mission Intelligence</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Harmattan AI</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4446051565/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Flight Control &amp; Dynamics Engineer</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Harmattan AI</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4475347864/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Sales Director Government Programs EMEA</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Jet Aviation</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Basel, Basel, Switzerland</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Government &amp; Special Mission Programs (Verteidigung/Behörden)</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4471449605/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Team Leader Account Management</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Pilatus Aircraft Ltd</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Stans, Nidwalden, Switzerland</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Account Management für Government-Aviation-Kunden (Militär)</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4466805480/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Director Project House C5I</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>RUAG</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Thun, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4466236796/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Head of S&amp;C Ground Thun</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>RUAG</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Thun, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4469362716/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Project Manager Protection</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>RUAG</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Thun, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4466950011/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Project Manager UAV &amp; cUAV</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>RUAG</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Emmen, Lucerne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4473985550/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>Technician Avionics</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>RUAG</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Wilderswil, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4471220489/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Program Manager Mission System (Defense &amp; High-Tech Mobility)</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Randstad Switzerland</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Tägerwilen, Thurgau, Switzerland</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464798329/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Area Sales Manager (m/w/d)</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Rheinmetall</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464232531/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Leiter Logistik (m/w/d)</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Rheinmetall</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Altdorf, Uri, Switzerland</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4467181674/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Senior Project Manager Air Defence (m/w/d)</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Rheinmetall</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4467181676/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Skysec Defence</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Aadorf, Thurgau, Switzerland</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Firma Skysec Defence</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4472247311/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Anordnungskoordinator/-in Kommando Operationen</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Swiss Armed Forces</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Bern, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4464864502/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Consulente TIC professional</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Swiss Armed Forces</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Bern, Berne, Switzerland</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4465724721/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Radar-Controller/-in (Track Monitor)</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Swiss Armed Forces</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Dübendorf, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4473757212/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Business Developer Defense - 100%</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Tethys Robotics</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Schlieren, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4466651737/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Senior Embedded Software and Processing Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Thales</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4450725792/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Senior PCB-CCA Designer in Space Products (m/w/d)</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Thales</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Zurich, Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Rüstungsfirma oder Verteidigungsbezug im Titel</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4470969808/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Senior Project Manager (H/F)</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>fortil</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Geneva, Switzerland</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>Bereich 'Aeronautics &amp; Defense'</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4470914271/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId30"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>